<commit_message>
감사 수정 2026-06-10 13:36
</commit_message>
<xml_diff>
--- a/RNR_수입원가_2026_20260610.xlsx
+++ b/RNR_수입원가_2026_20260610.xlsx
@@ -433,7 +433,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="241">
+  <cellXfs count="245">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1125,6 +1125,18 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="10" fontId="20" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1209,6 +1221,13 @@
     <author>RNR 재무팀</author>
   </authors>
   <commentList>
+    <comment ref="S5" authorId="0" shapeId="0">
+      <text>
+        <t>관세율 0% 적용 (DHL 특송/인천세관 직통관)
+신고필증 미확보 - 면세 사유 확인 필요
+(신고번호 883504210357, 수리일 2025-09-05)</t>
+      </text>
+    </comment>
     <comment ref="S7" authorId="0" shapeId="0">
       <text>
         <t>ITA(정보기술협정) 관세면제
@@ -1285,6 +1304,34 @@
       <text>
         <t>ITA(정보기술협정) 관세면제
 HS 8518/8543 디지털시네마장비</t>
+      </text>
+    </comment>
+    <comment ref="S35" authorId="0" shapeId="0">
+      <text>
+        <t>ITA(정보기술협정) 관세면제
+HS 8543 — 디지털시네마 서버/IMB
+(정보기술협정 양허품목)</t>
+      </text>
+    </comment>
+    <comment ref="S37" authorId="0" shapeId="0">
+      <text>
+        <t>ITA(정보기술협정) 관세면제
+HS 8543 — 디지털시네마 서버/IMB
+(정보기술협정 양허품목)</t>
+      </text>
+    </comment>
+    <comment ref="S38" authorId="0" shapeId="0">
+      <text>
+        <t>ITA(정보기술협정) 관세면제
+HS 8543 — 디지털시네마 서버/IMB
+(정보기술협정 양허품목)</t>
+      </text>
+    </comment>
+    <comment ref="S62" authorId="0" shapeId="0">
+      <text>
+        <t>관세율 0.00% - 세율구분 C(가가, WTO/ITA 양허)
+수리반환 재수입 건, 부가세만 과세
+(신고필증 2235626351613M)</t>
       </text>
     </comment>
   </commentList>
@@ -4296,10 +4343,8 @@
       <c r="F24" s="174" t="n">
         <v>46080</v>
       </c>
-      <c r="G24" s="175" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G24" s="175" t="n">
+        <v>46126</v>
       </c>
       <c r="H24" s="7" t="n">
         <v>36190</v>
@@ -4429,10 +4474,8 @@
       <c r="F25" s="174" t="n">
         <v>46088</v>
       </c>
-      <c r="G25" s="175" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G25" s="175" t="n">
+        <v>46126</v>
       </c>
       <c r="H25" s="7" t="n">
         <v>180</v>
@@ -4562,10 +4605,8 @@
       <c r="F26" s="174" t="n">
         <v>46088</v>
       </c>
-      <c r="G26" s="175" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G26" s="175" t="n">
+        <v>46126</v>
       </c>
       <c r="H26" s="7" t="n">
         <v>21280</v>
@@ -4957,7 +4998,9 @@
       <c r="F29" s="174" t="n">
         <v>46106</v>
       </c>
-      <c r="G29" s="175" t="n"/>
+      <c r="G29" s="175" t="n">
+        <v>46162</v>
+      </c>
       <c r="H29" s="7" t="n">
         <v>4290</v>
       </c>
@@ -5072,10 +5115,8 @@
       <c r="F30" s="179" t="n">
         <v>46113</v>
       </c>
-      <c r="G30" s="179" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G30" s="179" t="n">
+        <v>46171</v>
       </c>
       <c r="H30" s="80" t="n">
         <v>78209</v>
@@ -5193,10 +5234,8 @@
       <c r="F31" s="179" t="n">
         <v>46113</v>
       </c>
-      <c r="G31" s="179" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G31" s="179" t="n">
+        <v>46171</v>
       </c>
       <c r="H31" s="80" t="n">
         <v>8140</v>
@@ -5499,7 +5538,11 @@
         <f>ROUND(AA33/AB33,0)</f>
         <v/>
       </c>
-      <c r="AD33" s="129" t="n"/>
+      <c r="AD33" s="129" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
       <c r="AE33" s="129" t="n"/>
       <c r="AF33" s="129" t="n"/>
     </row>
@@ -5612,7 +5655,11 @@
         <f>ROUND(AA34/AB34,0)</f>
         <v/>
       </c>
-      <c r="AD34" s="129" t="n"/>
+      <c r="AD34" s="129" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
       <c r="AE34" s="129" t="n"/>
       <c r="AF34" s="129" t="n"/>
     </row>
@@ -5643,10 +5690,8 @@
       <c r="F35" s="181" t="n">
         <v>46113</v>
       </c>
-      <c r="G35" s="124" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G35" s="181" t="n">
+        <v>46171</v>
       </c>
       <c r="H35" s="126" t="n">
         <v>98800</v>
@@ -5725,7 +5770,11 @@
         <f>ROUND(AA35/AB35,0)</f>
         <v/>
       </c>
-      <c r="AD35" s="129" t="n"/>
+      <c r="AD35" s="129" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
       <c r="AE35" s="129" t="n"/>
       <c r="AF35" s="129" t="n"/>
     </row>
@@ -5756,10 +5805,8 @@
       <c r="F36" s="181" t="n">
         <v>46127</v>
       </c>
-      <c r="G36" s="124" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G36" s="181" t="n">
+        <v>46171</v>
       </c>
       <c r="H36" s="126" t="n">
         <v>90</v>
@@ -8328,10 +8375,8 @@
       <c r="F56" s="186" t="n">
         <v>46136</v>
       </c>
-      <c r="G56" s="186" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G56" s="186" t="n">
+        <v>46171</v>
       </c>
       <c r="H56" s="87" t="n">
         <v>15289</v>
@@ -8421,8 +8466,12 @@
           <t>2026-04</t>
         </is>
       </c>
-      <c r="AE56" s="186" t="n"/>
-      <c r="AF56" s="186" t="n"/>
+      <c r="AE56" s="186" t="n">
+        <v>46168</v>
+      </c>
+      <c r="AF56" s="186" t="n">
+        <v>46532</v>
+      </c>
     </row>
     <row r="57" ht="15.75" customHeight="1">
       <c r="A57" s="85" t="n">
@@ -8544,8 +8593,12 @@
           <t>2026-04</t>
         </is>
       </c>
-      <c r="AE57" s="186" t="n"/>
-      <c r="AF57" s="186" t="n"/>
+      <c r="AE57" s="186" t="n">
+        <v>46142</v>
+      </c>
+      <c r="AF57" s="186" t="n">
+        <v>46872</v>
+      </c>
     </row>
     <row r="58" ht="15.75" customHeight="1">
       <c r="A58" s="132" t="n">
@@ -8574,10 +8627,8 @@
       <c r="F58" s="188" t="n">
         <v>46127</v>
       </c>
-      <c r="G58" s="132" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G58" s="188" t="n">
+        <v>46161</v>
       </c>
       <c r="H58" s="134" t="n">
         <v>180</v>
@@ -8646,7 +8697,11 @@
         <f>ROUND(AA58/AB58,0)</f>
         <v/>
       </c>
-      <c r="AD58" s="137" t="n"/>
+      <c r="AD58" s="137" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
       <c r="AE58" s="189" t="n">
         <v>46143</v>
       </c>
@@ -8681,10 +8736,8 @@
       <c r="F59" s="188" t="n">
         <v>46137</v>
       </c>
-      <c r="G59" s="132" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G59" s="188" t="n">
+        <v>46171</v>
       </c>
       <c r="H59" s="134" t="n">
         <v>250</v>
@@ -8753,9 +8806,17 @@
         <f>ROUND(AA59/AB59,0)</f>
         <v/>
       </c>
-      <c r="AD59" s="137" t="n"/>
-      <c r="AE59" s="137" t="n"/>
-      <c r="AF59" s="137" t="n"/>
+      <c r="AD59" s="137" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="AE59" s="189" t="n">
+        <v>46143</v>
+      </c>
+      <c r="AF59" s="189" t="n">
+        <v>49795</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="132" t="n">
@@ -8859,8 +8920,16 @@
           <t>2026-06</t>
         </is>
       </c>
-      <c r="AE60" s="137" t="n"/>
-      <c r="AF60" s="137" t="n"/>
+      <c r="AE60" s="137" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF60" s="137" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="12" t="n">
@@ -9020,7 +9089,11 @@
         </is>
       </c>
       <c r="F62" s="176" t="n"/>
-      <c r="G62" s="177" t="n"/>
+      <c r="G62" s="177" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="H62" s="16" t="n">
         <v>400</v>
       </c>
@@ -10422,7 +10495,7 @@
       </c>
       <c r="K15" s="20" t="inlineStr">
         <is>
-          <t>홀딩</t>
+          <t>라이센스</t>
         </is>
       </c>
       <c r="L15" s="115" t="n"/>
@@ -10603,10 +10676,8 @@
       <c r="G19" s="184" t="n">
         <v>46109</v>
       </c>
-      <c r="H19" s="20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="H19" s="184" t="n">
+        <v>46146</v>
       </c>
       <c r="I19" s="184" t="n">
         <v>46113</v>
@@ -10652,10 +10723,8 @@
       <c r="G20" s="191" t="n">
         <v>46136</v>
       </c>
-      <c r="H20" s="191" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="H20" s="191" t="n">
+        <v>46171</v>
       </c>
       <c r="I20" s="191" t="n">
         <v>46168</v>
@@ -10750,10 +10819,8 @@
       <c r="G22" s="227" t="n">
         <v>46127</v>
       </c>
-      <c r="H22" s="227" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="H22" s="227" t="n">
+        <v>46161</v>
       </c>
       <c r="I22" s="227" t="n">
         <v>46143</v>
@@ -10799,10 +10866,8 @@
       <c r="G23" s="227" t="n">
         <v>46137</v>
       </c>
-      <c r="H23" s="227" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="H23" s="227" t="n">
+        <v>46171</v>
       </c>
       <c r="I23" s="227" t="n">
         <v>46143</v>
@@ -12143,6 +12208,270 @@
       <c r="K29" s="115" t="n"/>
       <c r="L29" s="115" t="n"/>
       <c r="M29" s="115" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="241" t="inlineStr">
+        <is>
+          <t>14008-26-101140M</t>
+        </is>
+      </c>
+      <c r="B30" s="241" t="inlineStr">
+        <is>
+          <t>CPO696-3</t>
+        </is>
+      </c>
+      <c r="C30" s="242" t="n">
+        <v>351274</v>
+      </c>
+      <c r="D30" s="243">
+        <f>C30/C30</f>
+        <v/>
+      </c>
+      <c r="E30" s="241" t="inlineStr">
+        <is>
+          <t>조운관세사무소</t>
+        </is>
+      </c>
+      <c r="F30" s="244" t="n">
+        <v>250000</v>
+      </c>
+      <c r="G30" s="241" t="inlineStr">
+        <is>
+          <t>조운관세사무소</t>
+        </is>
+      </c>
+      <c r="H30" s="244" t="n">
+        <v>3103207</v>
+      </c>
+      <c r="I30" s="241" t="inlineStr">
+        <is>
+          <t>단독</t>
+        </is>
+      </c>
+      <c r="J30" s="241" t="n"/>
+      <c r="K30" s="228" t="n"/>
+      <c r="L30" s="228" t="n"/>
+      <c r="M30" s="228" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="241" t="inlineStr">
+        <is>
+          <t>14008-26-101148M</t>
+        </is>
+      </c>
+      <c r="B31" s="241" t="inlineStr">
+        <is>
+          <t>GPO473-1</t>
+        </is>
+      </c>
+      <c r="C31" s="242" t="n">
+        <v>98800</v>
+      </c>
+      <c r="D31" s="243">
+        <f>C31/C31</f>
+        <v/>
+      </c>
+      <c r="E31" s="241" t="inlineStr">
+        <is>
+          <t>조운관세사무소</t>
+        </is>
+      </c>
+      <c r="F31" s="244" t="n">
+        <v>250000</v>
+      </c>
+      <c r="G31" s="241" t="inlineStr">
+        <is>
+          <t>조운관세사무소</t>
+        </is>
+      </c>
+      <c r="H31" s="244" t="n">
+        <v>3636072</v>
+      </c>
+      <c r="I31" s="241" t="inlineStr">
+        <is>
+          <t>단독</t>
+        </is>
+      </c>
+      <c r="J31" s="241" t="n"/>
+      <c r="K31" s="228" t="n"/>
+      <c r="L31" s="228" t="n"/>
+      <c r="M31" s="228" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="241" t="inlineStr">
+        <is>
+          <t>14008-26-101168M</t>
+        </is>
+      </c>
+      <c r="B32" s="241" t="inlineStr">
+        <is>
+          <t>CPO696-4</t>
+        </is>
+      </c>
+      <c r="C32" s="242" t="n">
+        <v>807233</v>
+      </c>
+      <c r="D32" s="243">
+        <f>C32/C32</f>
+        <v/>
+      </c>
+      <c r="E32" s="241" t="inlineStr">
+        <is>
+          <t>조운관세사무소</t>
+        </is>
+      </c>
+      <c r="F32" s="244" t="n">
+        <v>250000</v>
+      </c>
+      <c r="G32" s="241" t="inlineStr">
+        <is>
+          <t>조운관세사무소</t>
+        </is>
+      </c>
+      <c r="H32" s="244" t="n">
+        <v>3270326</v>
+      </c>
+      <c r="I32" s="241" t="inlineStr">
+        <is>
+          <t>단독</t>
+        </is>
+      </c>
+      <c r="J32" s="241" t="n"/>
+      <c r="K32" s="228" t="n"/>
+      <c r="L32" s="228" t="n"/>
+      <c r="M32" s="228" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="241" t="inlineStr">
+        <is>
+          <t>883504210357</t>
+        </is>
+      </c>
+      <c r="B33" s="241" t="inlineStr">
+        <is>
+          <t>IPO016</t>
+        </is>
+      </c>
+      <c r="C33" s="242" t="n">
+        <v>6800</v>
+      </c>
+      <c r="D33" s="243">
+        <f>C33/C33</f>
+        <v/>
+      </c>
+      <c r="E33" s="241" t="inlineStr">
+        <is>
+          <t>인천세관(특송)</t>
+        </is>
+      </c>
+      <c r="F33" s="244" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="241" t="inlineStr">
+        <is>
+          <t>DHL</t>
+        </is>
+      </c>
+      <c r="H33" s="244" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" s="241" t="inlineStr">
+        <is>
+          <t>단독</t>
+        </is>
+      </c>
+      <c r="J33" s="241" t="n"/>
+      <c r="K33" s="228" t="n"/>
+      <c r="L33" s="228" t="n"/>
+      <c r="M33" s="228" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="241" t="inlineStr">
+        <is>
+          <t>22356-26-351613M</t>
+        </is>
+      </c>
+      <c r="B34" s="241" t="inlineStr">
+        <is>
+          <t>SX3000수리</t>
+        </is>
+      </c>
+      <c r="C34" s="242" t="n">
+        <v>400</v>
+      </c>
+      <c r="D34" s="243">
+        <f>C34/C34</f>
+        <v/>
+      </c>
+      <c r="E34" s="241" t="inlineStr">
+        <is>
+          <t>운서합동관세사무소</t>
+        </is>
+      </c>
+      <c r="F34" s="244" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="241" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H34" s="244" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="241" t="inlineStr">
+        <is>
+          <t>단독</t>
+        </is>
+      </c>
+      <c r="J34" s="241" t="n"/>
+      <c r="K34" s="228" t="n"/>
+      <c r="L34" s="228" t="n"/>
+      <c r="M34" s="228" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="241" t="inlineStr">
+        <is>
+          <t>2235626346781M</t>
+        </is>
+      </c>
+      <c r="B35" s="241" t="inlineStr">
+        <is>
+          <t>CPO698</t>
+        </is>
+      </c>
+      <c r="C35" s="242" t="n">
+        <v>4290</v>
+      </c>
+      <c r="D35" s="243">
+        <f>C35/C35</f>
+        <v/>
+      </c>
+      <c r="E35" s="241" t="inlineStr">
+        <is>
+          <t>운서합동관세사무소</t>
+        </is>
+      </c>
+      <c r="F35" s="244" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="241" t="inlineStr">
+        <is>
+          <t>DHL</t>
+        </is>
+      </c>
+      <c r="H35" s="244" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" s="241" t="inlineStr">
+        <is>
+          <t>단독</t>
+        </is>
+      </c>
+      <c r="J35" s="241" t="n"/>
+      <c r="K35" s="228" t="n"/>
+      <c r="L35" s="228" t="n"/>
+      <c r="M35" s="228" t="n"/>
     </row>
     <row r="71">
       <c r="M71" s="40" t="n"/>

</xml_diff>

<commit_message>
5월 운송료 반영 2026-06-10 13:46
</commit_message>
<xml_diff>
--- a/RNR_수입원가_2026_20260610.xlsx
+++ b/RNR_수입원가_2026_20260610.xlsx
@@ -1306,6 +1306,12 @@
 HS 8518/8543 디지털시네마장비</t>
       </text>
     </comment>
+    <comment ref="Y29" authorId="0" shapeId="0">
+      <text>
+        <t>DHL 2026-05월 인보이스 (AWB 2538226250, 4/8 Christie HK 발송)
+지출결의 2026-1344, 6/9 집행</t>
+      </text>
+    </comment>
     <comment ref="S35" authorId="0" shapeId="0">
       <text>
         <t>ITA(정보기술협정) 관세면제
@@ -1327,11 +1333,24 @@
 (정보기술협정 양허품목)</t>
       </text>
     </comment>
-    <comment ref="S62" authorId="0" shapeId="0">
+    <comment ref="Y39" authorId="0" shapeId="0">
+      <text>
+        <t>FedEx 2026-05월 인보이스 159,250원 선반영
+(AWB 870900398456, 4/21 INTEG 발송, 4/27 배달)
+인보이스/송금/수입신고 미도래 - 미확정 건</t>
+      </text>
+    </comment>
+    <comment ref="S63" authorId="0" shapeId="0">
       <text>
         <t>관세율 0.00% - 세율구분 C(가가, WTO/ITA 양허)
 수리반환 재수입 건, 부가세만 과세
 (신고필증 2235626351613M)</t>
+      </text>
+    </comment>
+    <comment ref="Y63" authorId="0" shapeId="0">
+      <text>
+        <t>DHL 2026-05월 인보이스 (AWB 5094871784 = 수입신고필증 B/L 일치)
+GDC RMA 수리반환 건, 지출결의 2026-1344, 6/9 집행</t>
       </text>
     </comment>
   </commentList>
@@ -1552,7 +1571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF86"/>
+  <dimension ref="A1:AF87"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="17"/>
   <cols>
     <col width="5" customWidth="1" style="160" min="1" max="1"/>
@@ -5063,7 +5082,7 @@
         </is>
       </c>
       <c r="Y29" s="9" t="n">
-        <v>0</v>
+        <v>174806</v>
       </c>
       <c r="Z29" s="9">
         <f>S29+T29+W29</f>
@@ -6118,175 +6137,165 @@
       <c r="AF38" s="208" t="n"/>
     </row>
     <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="20" t="n">
-        <v>29</v>
-      </c>
-      <c r="B39" s="20" t="inlineStr">
-        <is>
-          <t>CPO667</t>
-        </is>
-      </c>
-      <c r="C39" s="21" t="inlineStr">
-        <is>
-          <t>Christie</t>
-        </is>
-      </c>
-      <c r="D39" s="20" t="inlineStr">
-        <is>
-          <t>Net 45 days</t>
-        </is>
-      </c>
-      <c r="E39" s="21" t="inlineStr">
-        <is>
-          <t>워런티(EW)</t>
-        </is>
-      </c>
-      <c r="F39" s="183" t="n">
-        <v>45925</v>
-      </c>
-      <c r="G39" s="184" t="n">
-        <v>46080</v>
-      </c>
-      <c r="H39" s="24" t="n">
-        <v>5673</v>
-      </c>
-      <c r="I39" s="185">
+      <c r="A39" s="124" t="n">
+        <v>60</v>
+      </c>
+      <c r="B39" s="124" t="inlineStr">
+        <is>
+          <t>IPO017</t>
+        </is>
+      </c>
+      <c r="C39" s="124" t="inlineStr">
+        <is>
+          <t>Integ Process Group</t>
+        </is>
+      </c>
+      <c r="D39" s="124" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E39" s="124" t="inlineStr">
+        <is>
+          <t>부품</t>
+        </is>
+      </c>
+      <c r="F39" s="181" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G39" s="181" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H39" s="126" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" s="126">
         <f>IFERROR(VLOOKUP(B39,RemitTable2,7,FALSE),0)</f>
         <v/>
       </c>
-      <c r="J39" s="26" t="n">
-        <v>205028994</v>
-      </c>
-      <c r="K39" s="26">
+      <c r="J39" s="128" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" s="128">
         <f>IFERROR(ROUND(H39*I39,0),0)</f>
         <v/>
       </c>
-      <c r="L39" s="26">
+      <c r="L39" s="128">
         <f>IFERROR(VLOOKUP(B39,RemitTable2,10,FALSE),0)</f>
         <v/>
       </c>
-      <c r="M39" s="26">
+      <c r="M39" s="128">
         <f>IFERROR(VLOOKUP(B39,RemitTable2,11,FALSE),0)</f>
         <v/>
       </c>
-      <c r="N39" s="20" t="inlineStr">
-        <is>
-          <t>EW CP2220</t>
-        </is>
-      </c>
-      <c r="O39" s="20" t="inlineStr">
+      <c r="N39" s="129" t="inlineStr">
+        <is>
+          <t>JNIOR Model 410 (IPO017, FedEx 4/21 발송분)</t>
+        </is>
+      </c>
+      <c r="O39" s="129" t="n"/>
+      <c r="P39" s="129" t="n"/>
+      <c r="Q39" s="126">
+        <f>IF(P39="","",IFERROR(VLOOKUP(O39,FxRateTable,4,TRUE),""))</f>
+        <v/>
+      </c>
+      <c r="R39" s="126">
+        <f>IF(P39="","",H39)</f>
+        <v/>
+      </c>
+      <c r="S39" s="128" t="n">
+        <v>0</v>
+      </c>
+      <c r="T39" s="128" t="n">
+        <v>0</v>
+      </c>
+      <c r="U39" s="129" t="n"/>
+      <c r="V39" s="129" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="P39" s="20" t="inlineStr">
+      <c r="W39" s="128" t="n">
+        <v>0</v>
+      </c>
+      <c r="X39" s="124" t="inlineStr">
+        <is>
+          <t>FedEx</t>
+        </is>
+      </c>
+      <c r="Y39" s="128" t="n">
+        <v>159250</v>
+      </c>
+      <c r="Z39" s="128">
+        <f>S39+T39+W39</f>
+        <v/>
+      </c>
+      <c r="AA39" s="131">
+        <f>K39+L39+M39+IFERROR(VLOOKUP(B39,RemitTable2,9,FALSE),0)+Y39+Z39</f>
+        <v/>
+      </c>
+      <c r="AB39" s="167" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC39" s="131">
+        <f>ROUND(AA39/AB39,0)</f>
+        <v/>
+      </c>
+      <c r="AD39" s="129" t="n"/>
+      <c r="AE39" s="129" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="Q39" s="24">
-        <f>IF(P39="","",IFERROR(VLOOKUP(O39,FxRateTable,4,TRUE),""))</f>
-        <v/>
-      </c>
-      <c r="R39" s="26">
-        <f>IF(P39="","",H39)</f>
-        <v/>
-      </c>
-      <c r="S39" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="T39" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="U39" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="V39" s="20" t="inlineStr">
+      <c r="AF39" s="129" t="inlineStr">
         <is>
           <t>-</t>
-        </is>
-      </c>
-      <c r="W39" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="X39" s="21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y39" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z39" s="26">
-        <f>S39+T39+W39</f>
-        <v/>
-      </c>
-      <c r="AA39" s="26">
-        <f>K39+L39+M39+IFERROR(VLOOKUP(B39,RemitTable2,9,FALSE),0)+Y39+Z39</f>
-        <v/>
-      </c>
-      <c r="AB39" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC39" s="26">
-        <f>ROUND(AA39/AB39,0)</f>
-        <v/>
-      </c>
-      <c r="AD39" s="20" t="inlineStr">
-        <is>
-          <t>2025-09</t>
-        </is>
-      </c>
-      <c r="AE39" s="184" t="inlineStr">
-        <is>
-          <t>2025-09-13</t>
-        </is>
-      </c>
-      <c r="AF39" s="183" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
         </is>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="20" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B40" s="20" t="inlineStr">
         <is>
-          <t>GPO458</t>
+          <t>CPO667</t>
         </is>
       </c>
       <c r="C40" s="21" t="inlineStr">
         <is>
-          <t>GDC</t>
+          <t>Christie</t>
         </is>
       </c>
       <c r="D40" s="20" t="inlineStr">
         <is>
-          <t>Net 30 days</t>
+          <t>Net 45 days</t>
         </is>
       </c>
       <c r="E40" s="21" t="inlineStr">
         <is>
-          <t>라이센스</t>
+          <t>워런티(EW)</t>
         </is>
       </c>
       <c r="F40" s="183" t="n">
-        <v>45982</v>
+        <v>45925</v>
       </c>
       <c r="G40" s="184" t="n">
-        <v>46020</v>
+        <v>46080</v>
       </c>
       <c r="H40" s="24" t="n">
-        <v>350</v>
+        <v>5673</v>
       </c>
       <c r="I40" s="185">
         <f>IFERROR(VLOOKUP(B40,RemitTable2,7,FALSE),0)</f>
         <v/>
       </c>
       <c r="J40" s="26" t="n">
-        <v>18264679</v>
+        <v>205028994</v>
       </c>
       <c r="K40" s="26">
         <f>IFERROR(ROUND(H40*I40,0),0)</f>
@@ -6302,7 +6311,7 @@
       </c>
       <c r="N40" s="20" t="inlineStr">
         <is>
-          <t>HFR License</t>
+          <t>EW CP2220</t>
         </is>
       </c>
       <c r="O40" s="20" t="inlineStr">
@@ -6365,59 +6374,59 @@
       </c>
       <c r="AD40" s="20" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2025-09</t>
         </is>
       </c>
       <c r="AE40" s="184" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-09-13</t>
         </is>
       </c>
       <c r="AF40" s="183" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="20" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B41" s="20" t="inlineStr">
         <is>
-          <t>CPO681</t>
+          <t>GPO458</t>
         </is>
       </c>
       <c r="C41" s="21" t="inlineStr">
         <is>
-          <t>Christie</t>
+          <t>GDC</t>
         </is>
       </c>
       <c r="D41" s="20" t="inlineStr">
         <is>
-          <t>Net 45 days</t>
+          <t>Net 30 days</t>
         </is>
       </c>
       <c r="E41" s="21" t="inlineStr">
         <is>
-          <t>워런티(EW)</t>
+          <t>라이센스</t>
         </is>
       </c>
       <c r="F41" s="183" t="n">
-        <v>45993</v>
+        <v>45982</v>
       </c>
       <c r="G41" s="184" t="n">
-        <v>46064</v>
+        <v>46020</v>
       </c>
       <c r="H41" s="24" t="n">
-        <v>26358</v>
+        <v>350</v>
       </c>
       <c r="I41" s="185">
         <f>IFERROR(VLOOKUP(B41,RemitTable2,7,FALSE),0)</f>
         <v/>
       </c>
       <c r="J41" s="26" t="n">
-        <v>38550844</v>
+        <v>18264679</v>
       </c>
       <c r="K41" s="26">
         <f>IFERROR(ROUND(H41*I41,0),0)</f>
@@ -6433,7 +6442,7 @@
       </c>
       <c r="N41" s="20" t="inlineStr">
         <is>
-          <t>EW CP2309/2315/2320-RGB</t>
+          <t>HFR License</t>
         </is>
       </c>
       <c r="O41" s="20" t="inlineStr">
@@ -6501,32 +6510,32 @@
       </c>
       <c r="AE41" s="184" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="AF41" s="183" t="inlineStr">
         <is>
-          <t>2026-12-21</t>
+          <t>2026-11-30</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="20" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B42" s="20" t="inlineStr">
         <is>
-          <t>GPO459</t>
+          <t>CPO681</t>
         </is>
       </c>
       <c r="C42" s="21" t="inlineStr">
         <is>
-          <t>GDC</t>
+          <t>Christie</t>
         </is>
       </c>
       <c r="D42" s="20" t="inlineStr">
         <is>
-          <t>Net 30 days</t>
+          <t>Net 45 days</t>
         </is>
       </c>
       <c r="E42" s="21" t="inlineStr">
@@ -6535,20 +6544,20 @@
         </is>
       </c>
       <c r="F42" s="183" t="n">
-        <v>46007</v>
+        <v>45993</v>
       </c>
       <c r="G42" s="184" t="n">
-        <v>46043</v>
+        <v>46064</v>
       </c>
       <c r="H42" s="24" t="n">
-        <v>450</v>
+        <v>26358</v>
       </c>
       <c r="I42" s="185">
         <f>IFERROR(VLOOKUP(B42,RemitTable2,7,FALSE),0)</f>
         <v/>
       </c>
       <c r="J42" s="26" t="n">
-        <v>5505104</v>
+        <v>38550844</v>
       </c>
       <c r="K42" s="26">
         <f>IFERROR(ROUND(H42*I42,0),0)</f>
@@ -6564,7 +6573,7 @@
       </c>
       <c r="N42" s="20" t="inlineStr">
         <is>
-          <t>TMS-2000 EW</t>
+          <t>EW CP2309/2315/2320-RGB</t>
         </is>
       </c>
       <c r="O42" s="20" t="inlineStr">
@@ -6627,27 +6636,27 @@
       </c>
       <c r="AD42" s="20" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="AE42" s="184" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="AF42" s="183" t="inlineStr">
         <is>
-          <t>2026-12-31</t>
+          <t>2026-12-21</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="20" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B43" s="20" t="inlineStr">
         <is>
-          <t>GPO461</t>
+          <t>GPO459</t>
         </is>
       </c>
       <c r="C43" s="21" t="inlineStr">
@@ -6672,7 +6681,7 @@
         <v>46043</v>
       </c>
       <c r="H43" s="24" t="n">
-        <v>540</v>
+        <v>450</v>
       </c>
       <c r="I43" s="185">
         <f>IFERROR(VLOOKUP(B43,RemitTable2,7,FALSE),0)</f>
@@ -6695,7 +6704,7 @@
       </c>
       <c r="N43" s="20" t="inlineStr">
         <is>
-          <t>TMS-1000 EW</t>
+          <t>TMS-2000 EW</t>
         </is>
       </c>
       <c r="O43" s="20" t="inlineStr">
@@ -6758,37 +6767,37 @@
       </c>
       <c r="AD43" s="20" t="inlineStr">
         <is>
-          <t>2025-11</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="AE43" s="184" t="inlineStr">
         <is>
-          <t>2025-11-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="AF43" s="183" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-12-31</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="20" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B44" s="20" t="inlineStr">
         <is>
-          <t>CPO685</t>
+          <t>GPO461</t>
         </is>
       </c>
       <c r="C44" s="21" t="inlineStr">
         <is>
-          <t>Christie</t>
+          <t>GDC</t>
         </is>
       </c>
       <c r="D44" s="20" t="inlineStr">
         <is>
-          <t>Net 45 days</t>
+          <t>Net 30 days</t>
         </is>
       </c>
       <c r="E44" s="21" t="inlineStr">
@@ -6797,20 +6806,20 @@
         </is>
       </c>
       <c r="F44" s="183" t="n">
-        <v>46010</v>
+        <v>46007</v>
       </c>
       <c r="G44" s="184" t="n">
-        <v>46080</v>
+        <v>46043</v>
       </c>
       <c r="H44" s="24" t="n">
-        <v>136516</v>
+        <v>540</v>
       </c>
       <c r="I44" s="185">
         <f>IFERROR(VLOOKUP(B44,RemitTable2,7,FALSE),0)</f>
         <v/>
       </c>
       <c r="J44" s="26" t="n">
-        <v>205028994</v>
+        <v>5505104</v>
       </c>
       <c r="K44" s="26">
         <f>IFERROR(ROUND(H44*I44,0),0)</f>
@@ -6826,7 +6835,7 @@
       </c>
       <c r="N44" s="20" t="inlineStr">
         <is>
-          <t>EW 대량 (CP2208~CP4450)</t>
+          <t>TMS-1000 EW</t>
         </is>
       </c>
       <c r="O44" s="20" t="inlineStr">
@@ -6889,37 +6898,37 @@
       </c>
       <c r="AD44" s="20" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2025-11</t>
         </is>
       </c>
       <c r="AE44" s="184" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2025-11-01</t>
         </is>
       </c>
       <c r="AF44" s="183" t="inlineStr">
         <is>
-          <t>2026-12-31</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="20" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B45" s="20" t="inlineStr">
         <is>
-          <t>GPO465</t>
+          <t>CPO685</t>
         </is>
       </c>
       <c r="C45" s="21" t="inlineStr">
         <is>
-          <t>GDC</t>
+          <t>Christie</t>
         </is>
       </c>
       <c r="D45" s="20" t="inlineStr">
         <is>
-          <t>Net 30 days</t>
+          <t>Net 45 days</t>
         </is>
       </c>
       <c r="E45" s="21" t="inlineStr">
@@ -6928,22 +6937,20 @@
         </is>
       </c>
       <c r="F45" s="183" t="n">
-        <v>46015</v>
-      </c>
-      <c r="G45" s="184" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>46010</v>
+      </c>
+      <c r="G45" s="184" t="n">
+        <v>46080</v>
       </c>
       <c r="H45" s="24" t="n">
-        <v>76054</v>
+        <v>136516</v>
       </c>
       <c r="I45" s="185">
         <f>IFERROR(VLOOKUP(B45,RemitTable2,7,FALSE),0)</f>
         <v/>
       </c>
       <c r="J45" s="26" t="n">
-        <v>0</v>
+        <v>205028994</v>
       </c>
       <c r="K45" s="26">
         <f>IFERROR(ROUND(H45*I45,0),0)</f>
@@ -6959,7 +6966,7 @@
       </c>
       <c r="N45" s="20" t="inlineStr">
         <is>
-          <t>EW 대량 (SR/SX/TMS)</t>
+          <t>EW 대량 (CP2208~CP4450)</t>
         </is>
       </c>
       <c r="O45" s="20" t="inlineStr">
@@ -7038,21 +7045,21 @@
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="20" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B46" s="20" t="inlineStr">
         <is>
-          <t>CPO686</t>
+          <t>GPO465</t>
         </is>
       </c>
       <c r="C46" s="21" t="inlineStr">
         <is>
-          <t>Christie</t>
+          <t>GDC</t>
         </is>
       </c>
       <c r="D46" s="20" t="inlineStr">
         <is>
-          <t>Net 45 days</t>
+          <t>Net 30 days</t>
         </is>
       </c>
       <c r="E46" s="21" t="inlineStr">
@@ -7061,20 +7068,22 @@
         </is>
       </c>
       <c r="F46" s="183" t="n">
-        <v>46029</v>
-      </c>
-      <c r="G46" s="184" t="n">
-        <v>46072</v>
+        <v>46015</v>
+      </c>
+      <c r="G46" s="184" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="H46" s="24" t="n">
-        <v>14793</v>
+        <v>76054</v>
       </c>
       <c r="I46" s="185">
         <f>IFERROR(VLOOKUP(B46,RemitTable2,7,FALSE),0)</f>
         <v/>
       </c>
       <c r="J46" s="26" t="n">
-        <v>25506948</v>
+        <v>0</v>
       </c>
       <c r="K46" s="26">
         <f>IFERROR(ROUND(H46*I46,0),0)</f>
@@ -7090,7 +7099,7 @@
       </c>
       <c r="N46" s="20" t="inlineStr">
         <is>
-          <t>EW CP2315/CP4440-RGB</t>
+          <t>EW 대량 (SR/SX/TMS)</t>
         </is>
       </c>
       <c r="O46" s="20" t="inlineStr">
@@ -7158,22 +7167,22 @@
       </c>
       <c r="AE46" s="184" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="AF46" s="183" t="inlineStr">
         <is>
-          <t>2027-01-29</t>
+          <t>2026-12-31</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="20" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B47" s="20" t="inlineStr">
         <is>
-          <t>CPO687</t>
+          <t>CPO686</t>
         </is>
       </c>
       <c r="C47" s="21" t="inlineStr">
@@ -7194,20 +7203,18 @@
       <c r="F47" s="183" t="n">
         <v>46029</v>
       </c>
-      <c r="G47" s="184" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G47" s="184" t="n">
+        <v>46072</v>
       </c>
       <c r="H47" s="24" t="n">
-        <v>26656</v>
+        <v>14793</v>
       </c>
       <c r="I47" s="185">
         <f>IFERROR(VLOOKUP(B47,RemitTable2,7,FALSE),0)</f>
         <v/>
       </c>
       <c r="J47" s="26" t="n">
-        <v>0</v>
+        <v>25506948</v>
       </c>
       <c r="K47" s="26">
         <f>IFERROR(ROUND(H47*I47,0),0)</f>
@@ -7223,7 +7230,7 @@
       </c>
       <c r="N47" s="20" t="inlineStr">
         <is>
-          <t>EW (홀딩)</t>
+          <t>EW CP2315/CP4440-RGB</t>
         </is>
       </c>
       <c r="O47" s="20" t="inlineStr">
@@ -7291,54 +7298,56 @@
       </c>
       <c r="AE47" s="184" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="AF47" s="183" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2027-01-29</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1">
       <c r="A48" s="20" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B48" s="20" t="inlineStr">
         <is>
-          <t>GPO462</t>
+          <t>CPO687</t>
         </is>
       </c>
       <c r="C48" s="21" t="inlineStr">
         <is>
-          <t>GDC</t>
+          <t>Christie</t>
         </is>
       </c>
       <c r="D48" s="20" t="inlineStr">
         <is>
-          <t>Net 30 days</t>
+          <t>Net 45 days</t>
         </is>
       </c>
       <c r="E48" s="21" t="inlineStr">
         <is>
-          <t>라이센스</t>
+          <t>워런티(EW)</t>
         </is>
       </c>
       <c r="F48" s="183" t="n">
-        <v>46042</v>
-      </c>
-      <c r="G48" s="184" t="n">
-        <v>46057</v>
+        <v>46029</v>
+      </c>
+      <c r="G48" s="184" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="H48" s="24" t="n">
-        <v>1440</v>
+        <v>26656</v>
       </c>
       <c r="I48" s="185">
         <f>IFERROR(VLOOKUP(B48,RemitTable2,7,FALSE),0)</f>
         <v/>
       </c>
       <c r="J48" s="26" t="n">
-        <v>16908206</v>
+        <v>0</v>
       </c>
       <c r="K48" s="26">
         <f>IFERROR(ROUND(H48*I48,0),0)</f>
@@ -7354,7 +7363,7 @@
       </c>
       <c r="N48" s="20" t="inlineStr">
         <is>
-          <t>TMS-2000 License</t>
+          <t>EW (홀딩)</t>
         </is>
       </c>
       <c r="O48" s="20" t="inlineStr">
@@ -7422,22 +7431,22 @@
       </c>
       <c r="AE48" s="184" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AF48" s="183" t="inlineStr">
         <is>
-          <t>2026-12-31</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="20" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B49" s="20" t="inlineStr">
         <is>
-          <t>GPO463</t>
+          <t>GPO462</t>
         </is>
       </c>
       <c r="C49" s="21" t="inlineStr">
@@ -7452,7 +7461,7 @@
       </c>
       <c r="E49" s="21" t="inlineStr">
         <is>
-          <t>워런티(EW)</t>
+          <t>라이센스</t>
         </is>
       </c>
       <c r="F49" s="183" t="n">
@@ -7462,7 +7471,7 @@
         <v>46057</v>
       </c>
       <c r="H49" s="24" t="n">
-        <v>4489</v>
+        <v>1440</v>
       </c>
       <c r="I49" s="185">
         <f>IFERROR(VLOOKUP(B49,RemitTable2,7,FALSE),0)</f>
@@ -7485,7 +7494,7 @@
       </c>
       <c r="N49" s="20" t="inlineStr">
         <is>
-          <t>SX/SR EW (CGV/Lotte)</t>
+          <t>TMS-2000 License</t>
         </is>
       </c>
       <c r="O49" s="20" t="inlineStr">
@@ -7564,11 +7573,11 @@
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="20" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B50" s="20" t="inlineStr">
         <is>
-          <t>GPO464</t>
+          <t>GPO463</t>
         </is>
       </c>
       <c r="C50" s="21" t="inlineStr">
@@ -7593,7 +7602,7 @@
         <v>46057</v>
       </c>
       <c r="H50" s="24" t="n">
-        <v>5670.57</v>
+        <v>4489</v>
       </c>
       <c r="I50" s="185">
         <f>IFERROR(VLOOKUP(B50,RemitTable2,7,FALSE),0)</f>
@@ -7616,7 +7625,7 @@
       </c>
       <c r="N50" s="20" t="inlineStr">
         <is>
-          <t>SR-1000/SX-3000 EW</t>
+          <t>SX/SR EW (CGV/Lotte)</t>
         </is>
       </c>
       <c r="O50" s="20" t="inlineStr">
@@ -7695,21 +7704,21 @@
     </row>
     <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="20" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B51" s="20" t="inlineStr">
         <is>
-          <t>CPO691</t>
+          <t>GPO464</t>
         </is>
       </c>
       <c r="C51" s="21" t="inlineStr">
         <is>
-          <t>Christie</t>
+          <t>GDC</t>
         </is>
       </c>
       <c r="D51" s="20" t="inlineStr">
         <is>
-          <t>Net 45 days</t>
+          <t>Net 30 days</t>
         </is>
       </c>
       <c r="E51" s="21" t="inlineStr">
@@ -7718,20 +7727,20 @@
         </is>
       </c>
       <c r="F51" s="183" t="n">
+        <v>46042</v>
+      </c>
+      <c r="G51" s="184" t="n">
         <v>46057</v>
       </c>
-      <c r="G51" s="184" t="n">
-        <v>46113</v>
-      </c>
       <c r="H51" s="24" t="n">
-        <v>24614</v>
+        <v>5670.57</v>
       </c>
       <c r="I51" s="185">
         <f>IFERROR(VLOOKUP(B51,RemitTable2,7,FALSE),0)</f>
         <v/>
       </c>
       <c r="J51" s="26" t="n">
-        <v>51777431</v>
+        <v>16908206</v>
       </c>
       <c r="K51" s="26">
         <f>IFERROR(ROUND(H51*I51,0),0)</f>
@@ -7747,7 +7756,7 @@
       </c>
       <c r="N51" s="20" t="inlineStr">
         <is>
-          <t>EW (메가박스 외)</t>
+          <t>SR-1000/SX-3000 EW</t>
         </is>
       </c>
       <c r="O51" s="20" t="inlineStr">
@@ -7810,37 +7819,37 @@
       </c>
       <c r="AD51" s="20" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="AE51" s="184" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="AF51" s="183" t="inlineStr">
         <is>
-          <t>2027-02-28</t>
+          <t>2026-12-31</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15.75" customHeight="1">
       <c r="A52" s="20" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B52" s="20" t="inlineStr">
         <is>
-          <t>GPO469</t>
+          <t>CPO691</t>
         </is>
       </c>
       <c r="C52" s="21" t="inlineStr">
         <is>
-          <t>GDC</t>
+          <t>Christie</t>
         </is>
       </c>
       <c r="D52" s="20" t="inlineStr">
         <is>
-          <t>Net 30 days</t>
+          <t>Net 45 days</t>
         </is>
       </c>
       <c r="E52" s="21" t="inlineStr">
@@ -7849,20 +7858,20 @@
         </is>
       </c>
       <c r="F52" s="183" t="n">
-        <v>46060</v>
+        <v>46057</v>
       </c>
       <c r="G52" s="184" t="n">
         <v>46113</v>
       </c>
       <c r="H52" s="24" t="n">
-        <v>3993.05</v>
+        <v>24614</v>
       </c>
       <c r="I52" s="185">
         <f>IFERROR(VLOOKUP(B52,RemitTable2,7,FALSE),0)</f>
         <v/>
       </c>
       <c r="J52" s="26" t="n">
-        <v>9919642</v>
+        <v>51777431</v>
       </c>
       <c r="K52" s="26">
         <f>IFERROR(ROUND(H52*I52,0),0)</f>
@@ -7878,7 +7887,7 @@
       </c>
       <c r="N52" s="20" t="inlineStr">
         <is>
-          <t>SR/SX EW (하남미사 외)</t>
+          <t>EW (메가박스 외)</t>
         </is>
       </c>
       <c r="O52" s="20" t="inlineStr">
@@ -7941,27 +7950,27 @@
       </c>
       <c r="AD52" s="20" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="AE52" s="184" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="AF52" s="183" t="inlineStr">
         <is>
-          <t>2027-02-22</t>
+          <t>2027-02-28</t>
         </is>
       </c>
     </row>
     <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="20" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B53" s="20" t="inlineStr">
         <is>
-          <t>GPO470</t>
+          <t>GPO469</t>
         </is>
       </c>
       <c r="C53" s="21" t="inlineStr">
@@ -7976,17 +7985,17 @@
       </c>
       <c r="E53" s="21" t="inlineStr">
         <is>
-          <t>라이센스</t>
+          <t>워런티(EW)</t>
         </is>
       </c>
       <c r="F53" s="183" t="n">
-        <v>46080</v>
+        <v>46060</v>
       </c>
       <c r="G53" s="184" t="n">
         <v>46113</v>
       </c>
       <c r="H53" s="24" t="n">
-        <v>360</v>
+        <v>3993.05</v>
       </c>
       <c r="I53" s="185">
         <f>IFERROR(VLOOKUP(B53,RemitTable2,7,FALSE),0)</f>
@@ -8009,7 +8018,7 @@
       </c>
       <c r="N53" s="20" t="inlineStr">
         <is>
-          <t>TMS-1000 License</t>
+          <t>SR/SX EW (하남미사 외)</t>
         </is>
       </c>
       <c r="O53" s="20" t="inlineStr">
@@ -8072,27 +8081,27 @@
       </c>
       <c r="AD53" s="20" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="AE53" s="184" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="AF53" s="183" t="inlineStr">
         <is>
-          <t>2027-02-28</t>
+          <t>2027-02-22</t>
         </is>
       </c>
     </row>
     <row r="54" ht="15.75" customHeight="1">
       <c r="A54" s="20" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B54" s="20" t="inlineStr">
         <is>
-          <t>GPO471</t>
+          <t>GPO470</t>
         </is>
       </c>
       <c r="C54" s="21" t="inlineStr">
@@ -8111,13 +8120,13 @@
         </is>
       </c>
       <c r="F54" s="183" t="n">
-        <v>46088</v>
+        <v>46080</v>
       </c>
       <c r="G54" s="184" t="n">
         <v>46113</v>
       </c>
       <c r="H54" s="24" t="n">
-        <v>500</v>
+        <v>360</v>
       </c>
       <c r="I54" s="185">
         <f>IFERROR(VLOOKUP(B54,RemitTable2,7,FALSE),0)</f>
@@ -8140,7 +8149,7 @@
       </c>
       <c r="N54" s="20" t="inlineStr">
         <is>
-          <t>Dolby Atmos License</t>
+          <t>TMS-1000 License</t>
         </is>
       </c>
       <c r="O54" s="20" t="inlineStr">
@@ -8208,54 +8217,54 @@
       </c>
       <c r="AE54" s="184" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="AF54" s="183" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2027-02-28</t>
         </is>
       </c>
     </row>
     <row r="55" ht="15.75" customHeight="1">
       <c r="A55" s="20" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B55" s="20" t="inlineStr">
         <is>
-          <t>CPO694</t>
+          <t>GPO471</t>
         </is>
       </c>
       <c r="C55" s="21" t="inlineStr">
         <is>
-          <t>Christie</t>
+          <t>GDC</t>
         </is>
       </c>
       <c r="D55" s="20" t="inlineStr">
         <is>
-          <t>Net 45 days</t>
+          <t>Net 30 days</t>
         </is>
       </c>
       <c r="E55" s="21" t="inlineStr">
         <is>
-          <t>워런티(EW)</t>
+          <t>라이센스</t>
         </is>
       </c>
       <c r="F55" s="183" t="n">
-        <v>46109</v>
+        <v>46088</v>
       </c>
       <c r="G55" s="184" t="n">
-        <v>46146</v>
+        <v>46113</v>
       </c>
       <c r="H55" s="24" t="n">
-        <v>17404</v>
+        <v>500</v>
       </c>
       <c r="I55" s="185">
         <f>IFERROR(VLOOKUP(B55,RemitTable2,7,FALSE),0)</f>
         <v/>
       </c>
       <c r="J55" s="26" t="n">
-        <v>0</v>
+        <v>9919642</v>
       </c>
       <c r="K55" s="26">
         <f>IFERROR(ROUND(H55*I55,0),0)</f>
@@ -8271,7 +8280,7 @@
       </c>
       <c r="N55" s="20" t="inlineStr">
         <is>
-          <t>EW (CGV 동백 외)</t>
+          <t>Dolby Atmos License</t>
         </is>
       </c>
       <c r="O55" s="20" t="inlineStr">
@@ -8334,152 +8343,158 @@
       </c>
       <c r="AD55" s="20" t="inlineStr">
         <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="AE55" s="184" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF55" s="183" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="15.75" customHeight="1">
+      <c r="A56" s="20" t="n">
+        <v>45</v>
+      </c>
+      <c r="B56" s="20" t="inlineStr">
+        <is>
+          <t>CPO694</t>
+        </is>
+      </c>
+      <c r="C56" s="21" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="D56" s="20" t="inlineStr">
+        <is>
+          <t>Net 45 days</t>
+        </is>
+      </c>
+      <c r="E56" s="21" t="inlineStr">
+        <is>
+          <t>워런티(EW)</t>
+        </is>
+      </c>
+      <c r="F56" s="183" t="n">
+        <v>46109</v>
+      </c>
+      <c r="G56" s="184" t="n">
+        <v>46146</v>
+      </c>
+      <c r="H56" s="24" t="n">
+        <v>17404</v>
+      </c>
+      <c r="I56" s="185">
+        <f>IFERROR(VLOOKUP(B56,RemitTable2,7,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="J56" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K56" s="26">
+        <f>IFERROR(ROUND(H56*I56,0),0)</f>
+        <v/>
+      </c>
+      <c r="L56" s="26">
+        <f>IFERROR(VLOOKUP(B56,RemitTable2,10,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="M56" s="26">
+        <f>IFERROR(VLOOKUP(B56,RemitTable2,11,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N56" s="20" t="inlineStr">
+        <is>
+          <t>EW (CGV 동백 외)</t>
+        </is>
+      </c>
+      <c r="O56" s="20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P56" s="20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q56" s="24">
+        <f>IF(P56="","",IFERROR(VLOOKUP(O56,FxRateTable,4,TRUE),""))</f>
+        <v/>
+      </c>
+      <c r="R56" s="26">
+        <f>IF(P56="","",H56)</f>
+        <v/>
+      </c>
+      <c r="S56" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="T56" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="U56" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="V56" s="20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W56" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="X56" s="21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y56" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z56" s="26">
+        <f>S56+T56+W56</f>
+        <v/>
+      </c>
+      <c r="AA56" s="26">
+        <f>K56+L56+M56+IFERROR(VLOOKUP(B56,RemitTable2,9,FALSE),0)+Y56+Z56</f>
+        <v/>
+      </c>
+      <c r="AB56" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC56" s="26">
+        <f>ROUND(AA56/AB56,0)</f>
+        <v/>
+      </c>
+      <c r="AD56" s="20" t="inlineStr">
+        <is>
           <t>2026-04</t>
         </is>
       </c>
-      <c r="AE55" s="184" t="inlineStr">
+      <c r="AE56" s="184" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="AF55" s="183" t="inlineStr">
+      <c r="AF56" s="183" t="inlineStr">
         <is>
           <t>2027-03-31</t>
         </is>
-      </c>
-    </row>
-    <row r="56" ht="15.75" customHeight="1">
-      <c r="A56" s="85" t="n">
-        <v>46</v>
-      </c>
-      <c r="B56" s="85" t="inlineStr">
-        <is>
-          <t>CPO697</t>
-        </is>
-      </c>
-      <c r="C56" s="85" t="inlineStr">
-        <is>
-          <t>Christie</t>
-        </is>
-      </c>
-      <c r="D56" s="85" t="inlineStr">
-        <is>
-          <t>Net 45 days</t>
-        </is>
-      </c>
-      <c r="E56" s="85" t="inlineStr">
-        <is>
-          <t>워런티(EW)</t>
-        </is>
-      </c>
-      <c r="F56" s="186" t="n">
-        <v>46136</v>
-      </c>
-      <c r="G56" s="186" t="n">
-        <v>46171</v>
-      </c>
-      <c r="H56" s="87" t="n">
-        <v>15289</v>
-      </c>
-      <c r="I56" s="187">
-        <f>IFERROR(VLOOKUP(B56,RemitTable2,7,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="J56" s="89" t="n">
-        <v>0</v>
-      </c>
-      <c r="K56" s="89">
-        <f>IFERROR(ROUND(H56*I56,0),0)</f>
-        <v/>
-      </c>
-      <c r="L56" s="89">
-        <f>IFERROR(VLOOKUP(B56,RemitTable2,10,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M56" s="89">
-        <f>IFERROR(VLOOKUP(B56,RemitTable2,11,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="N56" s="85" t="inlineStr">
-        <is>
-          <t>EW CP4425/CP2308/CP2315/CP2309/CP2320 13대 (메가박스 북대구 외)</t>
-        </is>
-      </c>
-      <c r="O56" s="186" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P56" s="85" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q56" s="87">
-        <f>IF(P56="","",IFERROR(VLOOKUP(O56,FxRateTable,4,TRUE),""))</f>
-        <v/>
-      </c>
-      <c r="R56" s="87">
-        <f>IF(P56="","",H56)</f>
-        <v/>
-      </c>
-      <c r="S56" s="89" t="n">
-        <v>0</v>
-      </c>
-      <c r="T56" s="89" t="n">
-        <v>0</v>
-      </c>
-      <c r="U56" s="186" t="n"/>
-      <c r="V56" s="85" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W56" s="89" t="n">
-        <v>0</v>
-      </c>
-      <c r="X56" s="85" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y56" s="89" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z56" s="89">
-        <f>S56+T56+W56</f>
-        <v/>
-      </c>
-      <c r="AA56" s="89">
-        <f>K56+L56+M56+IFERROR(VLOOKUP(B56,RemitTable2,9,FALSE),0)+Y56+Z56</f>
-        <v/>
-      </c>
-      <c r="AB56" s="90" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC56" s="89">
-        <f>ROUND(AA56/AB56,0)</f>
-        <v/>
-      </c>
-      <c r="AD56" s="85" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="AE56" s="186" t="n">
-        <v>46168</v>
-      </c>
-      <c r="AF56" s="186" t="n">
-        <v>46532</v>
       </c>
     </row>
     <row r="57" ht="15.75" customHeight="1">
       <c r="A57" s="85" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B57" s="85" t="inlineStr">
         <is>
-          <t>CPO693-2</t>
+          <t>CPO697</t>
         </is>
       </c>
       <c r="C57" s="85" t="inlineStr">
@@ -8498,15 +8513,13 @@
         </is>
       </c>
       <c r="F57" s="186" t="n">
-        <v>46133</v>
-      </c>
-      <c r="G57" s="186" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>46136</v>
+      </c>
+      <c r="G57" s="186" t="n">
+        <v>46171</v>
       </c>
       <c r="H57" s="87" t="n">
-        <v>2550</v>
+        <v>15289</v>
       </c>
       <c r="I57" s="187">
         <f>IFERROR(VLOOKUP(B57,RemitTable2,7,FALSE),0)</f>
@@ -8529,7 +8542,7 @@
       </c>
       <c r="N57" s="85" t="inlineStr">
         <is>
-          <t>CP4420-RGB 2년 워런티 (CGV 구미)</t>
+          <t>EW CP4425/CP2308/CP2315/CP2309/CP2320 13대 (메가박스 북대구 외)</t>
         </is>
       </c>
       <c r="O57" s="186" t="inlineStr">
@@ -8594,128 +8607,146 @@
         </is>
       </c>
       <c r="AE57" s="186" t="n">
+        <v>46168</v>
+      </c>
+      <c r="AF57" s="186" t="n">
+        <v>46532</v>
+      </c>
+    </row>
+    <row r="58" ht="15.75" customHeight="1">
+      <c r="A58" s="85" t="n">
+        <v>47</v>
+      </c>
+      <c r="B58" s="85" t="inlineStr">
+        <is>
+          <t>CPO693-2</t>
+        </is>
+      </c>
+      <c r="C58" s="85" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="D58" s="85" t="inlineStr">
+        <is>
+          <t>Net 45 days</t>
+        </is>
+      </c>
+      <c r="E58" s="85" t="inlineStr">
+        <is>
+          <t>워런티(EW)</t>
+        </is>
+      </c>
+      <c r="F58" s="186" t="n">
+        <v>46133</v>
+      </c>
+      <c r="G58" s="186" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H58" s="87" t="n">
+        <v>2550</v>
+      </c>
+      <c r="I58" s="187">
+        <f>IFERROR(VLOOKUP(B58,RemitTable2,7,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="J58" s="89" t="n">
+        <v>0</v>
+      </c>
+      <c r="K58" s="89">
+        <f>IFERROR(ROUND(H58*I58,0),0)</f>
+        <v/>
+      </c>
+      <c r="L58" s="89">
+        <f>IFERROR(VLOOKUP(B58,RemitTable2,10,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="M58" s="89">
+        <f>IFERROR(VLOOKUP(B58,RemitTable2,11,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N58" s="85" t="inlineStr">
+        <is>
+          <t>CP4420-RGB 2년 워런티 (CGV 구미)</t>
+        </is>
+      </c>
+      <c r="O58" s="186" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P58" s="85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q58" s="87">
+        <f>IF(P58="","",IFERROR(VLOOKUP(O58,FxRateTable,4,TRUE),""))</f>
+        <v/>
+      </c>
+      <c r="R58" s="87">
+        <f>IF(P58="","",H58)</f>
+        <v/>
+      </c>
+      <c r="S58" s="89" t="n">
+        <v>0</v>
+      </c>
+      <c r="T58" s="89" t="n">
+        <v>0</v>
+      </c>
+      <c r="U58" s="186" t="n"/>
+      <c r="V58" s="85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W58" s="89" t="n">
+        <v>0</v>
+      </c>
+      <c r="X58" s="85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y58" s="89" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z58" s="89">
+        <f>S58+T58+W58</f>
+        <v/>
+      </c>
+      <c r="AA58" s="89">
+        <f>K58+L58+M58+IFERROR(VLOOKUP(B58,RemitTable2,9,FALSE),0)+Y58+Z58</f>
+        <v/>
+      </c>
+      <c r="AB58" s="90" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC58" s="89">
+        <f>ROUND(AA58/AB58,0)</f>
+        <v/>
+      </c>
+      <c r="AD58" s="85" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="AE58" s="186" t="n">
         <v>46142</v>
       </c>
-      <c r="AF57" s="186" t="n">
+      <c r="AF58" s="186" t="n">
         <v>46872</v>
-      </c>
-    </row>
-    <row r="58" ht="15.75" customHeight="1">
-      <c r="A58" s="132" t="n">
-        <v>54</v>
-      </c>
-      <c r="B58" s="132" t="inlineStr">
-        <is>
-          <t>GPO478</t>
-        </is>
-      </c>
-      <c r="C58" s="132" t="inlineStr">
-        <is>
-          <t>GDC</t>
-        </is>
-      </c>
-      <c r="D58" s="132" t="inlineStr">
-        <is>
-          <t>Net 30 days</t>
-        </is>
-      </c>
-      <c r="E58" s="132" t="inlineStr">
-        <is>
-          <t>라이센스</t>
-        </is>
-      </c>
-      <c r="F58" s="188" t="n">
-        <v>46127</v>
-      </c>
-      <c r="G58" s="188" t="n">
-        <v>46161</v>
-      </c>
-      <c r="H58" s="134" t="n">
-        <v>180</v>
-      </c>
-      <c r="I58" s="134">
-        <f>IFERROR(VLOOKUP(B58,RemitTable2,7,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="J58" s="136" t="n">
-        <v>0</v>
-      </c>
-      <c r="K58" s="136">
-        <f>IFERROR(ROUND(H58*I58,0),0)</f>
-        <v/>
-      </c>
-      <c r="L58" s="136">
-        <f>IFERROR(VLOOKUP(B58,RemitTable2,10,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M58" s="136">
-        <f>IFERROR(VLOOKUP(B58,RemitTable2,11,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="N58" s="137" t="n"/>
-      <c r="O58" s="137" t="n"/>
-      <c r="P58" s="137" t="n"/>
-      <c r="Q58" s="134">
-        <f>IF(P58="","",IFERROR(VLOOKUP(O58,FxRateTable,4,TRUE),""))</f>
-        <v/>
-      </c>
-      <c r="R58" s="134">
-        <f>IF(P58="","",H58)</f>
-        <v/>
-      </c>
-      <c r="S58" s="136" t="n">
-        <v>0</v>
-      </c>
-      <c r="T58" s="136" t="n">
-        <v>0</v>
-      </c>
-      <c r="U58" s="137" t="n"/>
-      <c r="V58" s="137" t="n"/>
-      <c r="W58" s="136" t="n">
-        <v>0</v>
-      </c>
-      <c r="X58" s="132" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y58" s="136" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z58" s="136">
-        <f>S58+T58+W58</f>
-        <v/>
-      </c>
-      <c r="AA58" s="136">
-        <f>K58+L58+M58+IFERROR(VLOOKUP(B58,RemitTable2,9,FALSE),0)+Y58+Z58</f>
-        <v/>
-      </c>
-      <c r="AB58" s="168" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC58" s="136">
-        <f>ROUND(AA58/AB58,0)</f>
-        <v/>
-      </c>
-      <c r="AD58" s="137" t="inlineStr">
-        <is>
-          <t>2026-05</t>
-        </is>
-      </c>
-      <c r="AE58" s="189" t="n">
-        <v>46143</v>
-      </c>
-      <c r="AF58" s="189" t="n">
-        <v>46507</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="132" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B59" s="132" t="inlineStr">
         <is>
-          <t>GPO480</t>
+          <t>GPO478</t>
         </is>
       </c>
       <c r="C59" s="132" t="inlineStr">
@@ -8734,13 +8765,13 @@
         </is>
       </c>
       <c r="F59" s="188" t="n">
-        <v>46137</v>
+        <v>46127</v>
       </c>
       <c r="G59" s="188" t="n">
-        <v>46171</v>
+        <v>46161</v>
       </c>
       <c r="H59" s="134" t="n">
-        <v>250</v>
+        <v>180</v>
       </c>
       <c r="I59" s="134">
         <f>IFERROR(VLOOKUP(B59,RemitTable2,7,FALSE),0)</f>
@@ -8800,7 +8831,7 @@
         <v/>
       </c>
       <c r="AB59" s="168" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC59" s="136">
         <f>ROUND(AA59/AB59,0)</f>
@@ -8815,16 +8846,16 @@
         <v>46143</v>
       </c>
       <c r="AF59" s="189" t="n">
-        <v>49795</v>
+        <v>46507</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="132" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B60" s="132" t="inlineStr">
         <is>
-          <t>GPO481</t>
+          <t>GPO480</t>
         </is>
       </c>
       <c r="C60" s="132" t="inlineStr">
@@ -8843,13 +8874,13 @@
         </is>
       </c>
       <c r="F60" s="188" t="n">
-        <v>46152</v>
-      </c>
-      <c r="G60" s="233" t="n">
-        <v>46183</v>
+        <v>46137</v>
+      </c>
+      <c r="G60" s="188" t="n">
+        <v>46171</v>
       </c>
       <c r="H60" s="134" t="n">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="I60" s="134">
         <f>IFERROR(VLOOKUP(B60,RemitTable2,7,FALSE),0)</f>
@@ -8917,148 +8948,124 @@
       </c>
       <c r="AD60" s="137" t="inlineStr">
         <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="AE60" s="189" t="n">
+        <v>46143</v>
+      </c>
+      <c r="AF60" s="189" t="n">
+        <v>49795</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="132" t="n">
+        <v>56</v>
+      </c>
+      <c r="B61" s="132" t="inlineStr">
+        <is>
+          <t>GPO481</t>
+        </is>
+      </c>
+      <c r="C61" s="132" t="inlineStr">
+        <is>
+          <t>GDC</t>
+        </is>
+      </c>
+      <c r="D61" s="132" t="inlineStr">
+        <is>
+          <t>Net 30 days</t>
+        </is>
+      </c>
+      <c r="E61" s="132" t="inlineStr">
+        <is>
+          <t>라이센스</t>
+        </is>
+      </c>
+      <c r="F61" s="188" t="n">
+        <v>46152</v>
+      </c>
+      <c r="G61" s="233" t="n">
+        <v>46183</v>
+      </c>
+      <c r="H61" s="134" t="n">
+        <v>500</v>
+      </c>
+      <c r="I61" s="134">
+        <f>IFERROR(VLOOKUP(B61,RemitTable2,7,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="J61" s="136" t="n">
+        <v>0</v>
+      </c>
+      <c r="K61" s="136">
+        <f>IFERROR(ROUND(H61*I61,0),0)</f>
+        <v/>
+      </c>
+      <c r="L61" s="136">
+        <f>IFERROR(VLOOKUP(B61,RemitTable2,10,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="M61" s="136">
+        <f>IFERROR(VLOOKUP(B61,RemitTable2,11,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N61" s="137" t="n"/>
+      <c r="O61" s="137" t="n"/>
+      <c r="P61" s="137" t="n"/>
+      <c r="Q61" s="134">
+        <f>IF(P61="","",IFERROR(VLOOKUP(O61,FxRateTable,4,TRUE),""))</f>
+        <v/>
+      </c>
+      <c r="R61" s="134">
+        <f>IF(P61="","",H61)</f>
+        <v/>
+      </c>
+      <c r="S61" s="136" t="n">
+        <v>0</v>
+      </c>
+      <c r="T61" s="136" t="n">
+        <v>0</v>
+      </c>
+      <c r="U61" s="137" t="n"/>
+      <c r="V61" s="137" t="n"/>
+      <c r="W61" s="136" t="n">
+        <v>0</v>
+      </c>
+      <c r="X61" s="132" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y61" s="136" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z61" s="136">
+        <f>S61+T61+W61</f>
+        <v/>
+      </c>
+      <c r="AA61" s="136">
+        <f>K61+L61+M61+IFERROR(VLOOKUP(B61,RemitTable2,9,FALSE),0)+Y61+Z61</f>
+        <v/>
+      </c>
+      <c r="AB61" s="168" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC61" s="136">
+        <f>ROUND(AA61/AB61,0)</f>
+        <v/>
+      </c>
+      <c r="AD61" s="137" t="inlineStr">
+        <is>
           <t>2026-06</t>
         </is>
       </c>
-      <c r="AE60" s="137" t="inlineStr">
+      <c r="AE61" s="137" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AF60" s="137" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="12" t="n">
-        <v>48</v>
-      </c>
-      <c r="B61" s="12" t="inlineStr">
-        <is>
-          <t>CPO688</t>
-        </is>
-      </c>
-      <c r="C61" s="13" t="inlineStr">
-        <is>
-          <t>Christie</t>
-        </is>
-      </c>
-      <c r="D61" s="12" t="inlineStr">
-        <is>
-          <t>Net 45 days</t>
-        </is>
-      </c>
-      <c r="E61" s="13" t="inlineStr">
-        <is>
-          <t>Inspection</t>
-        </is>
-      </c>
-      <c r="F61" s="176" t="n">
-        <v>46037</v>
-      </c>
-      <c r="G61" s="177" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H61" s="16" t="n">
-        <v>4180</v>
-      </c>
-      <c r="I61" s="178">
-        <f>IFERROR(VLOOKUP(B61,RemitTable2,7,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="J61" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="K61" s="18">
-        <f>IFERROR(ROUND(H61*I61,0),0)</f>
-        <v/>
-      </c>
-      <c r="L61" s="18">
-        <f>IFERROR(VLOOKUP(B61,RemitTable2,10,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M61" s="18">
-        <f>IFERROR(VLOOKUP(B61,RemitTable2,11,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="N61" s="12" t="inlineStr">
-        <is>
-          <t>Inspection fee</t>
-        </is>
-      </c>
-      <c r="O61" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P61" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q61" s="16">
-        <f>IF(P61="","",IFERROR(VLOOKUP(O61,FxRateTable,4,TRUE),""))</f>
-        <v/>
-      </c>
-      <c r="R61" s="18">
-        <f>IF(P61="","",H61)</f>
-        <v/>
-      </c>
-      <c r="S61" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="T61" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="U61" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="V61" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W61" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="X61" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y61" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z61" s="18">
-        <f>S61+T61+W61</f>
-        <v/>
-      </c>
-      <c r="AA61" s="18">
-        <f>K61+L61+M61+IFERROR(VLOOKUP(B61,RemitTable2,9,FALSE),0)+Y61+Z61</f>
-        <v/>
-      </c>
-      <c r="AB61" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC61" s="18">
-        <f>ROUND(AA61/AB61,0)</f>
-        <v/>
-      </c>
-      <c r="AD61" s="12" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="AE61" s="177" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AF61" s="176" t="inlineStr">
+      <c r="AF61" s="137" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -9066,36 +9073,38 @@
     </row>
     <row r="62">
       <c r="A62" s="12" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B62" s="12" t="inlineStr">
         <is>
-          <t>SX3000수리</t>
+          <t>CPO688</t>
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr">
         <is>
-          <t>GDC</t>
+          <t>Christie</t>
         </is>
       </c>
       <c r="D62" s="12" t="inlineStr">
         <is>
+          <t>Net 45 days</t>
+        </is>
+      </c>
+      <c r="E62" s="13" t="inlineStr">
+        <is>
+          <t>Inspection</t>
+        </is>
+      </c>
+      <c r="F62" s="176" t="n">
+        <v>46037</v>
+      </c>
+      <c r="G62" s="177" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E62" s="13" t="inlineStr">
-        <is>
-          <t>수리반환</t>
-        </is>
-      </c>
-      <c r="F62" s="176" t="n"/>
-      <c r="G62" s="177" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="H62" s="16" t="n">
-        <v>400</v>
+        <v>4180</v>
       </c>
       <c r="I62" s="178">
         <f>IFERROR(VLOOKUP(B62,RemitTable2,7,FALSE),0)</f>
@@ -9118,15 +9127,17 @@
       </c>
       <c r="N62" s="12" t="inlineStr">
         <is>
-          <t>Display Card (수리반환 5PCS)</t>
-        </is>
-      </c>
-      <c r="O62" s="177" t="n">
-        <v>46125</v>
+          <t>Inspection fee</t>
+        </is>
+      </c>
+      <c r="O62" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="P62" s="12" t="inlineStr">
         <is>
-          <t>22356-26-351613M</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q62" s="16">
@@ -9141,12 +9152,14 @@
         <v>0</v>
       </c>
       <c r="T62" s="18" t="n">
-        <v>67750</v>
-      </c>
-      <c r="U62" s="13" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="U62" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="V62" s="12" t="inlineStr">
         <is>
-          <t>운서합동</t>
+          <t>-</t>
         </is>
       </c>
       <c r="W62" s="18" t="n">
@@ -9154,7 +9167,7 @@
       </c>
       <c r="X62" s="13" t="inlineStr">
         <is>
-          <t>DHL</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Y62" s="18" t="n">
@@ -9169,7 +9182,7 @@
         <v/>
       </c>
       <c r="AB62" s="19" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AC62" s="18">
         <f>ROUND(AA62/AB62,0)</f>
@@ -9177,206 +9190,262 @@
       </c>
       <c r="AD62" s="12" t="inlineStr">
         <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="AE62" s="177" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF62" s="176" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="12" t="n">
+        <v>49</v>
+      </c>
+      <c r="B63" s="12" t="inlineStr">
+        <is>
+          <t>SX3000수리</t>
+        </is>
+      </c>
+      <c r="C63" s="13" t="inlineStr">
+        <is>
+          <t>GDC</t>
+        </is>
+      </c>
+      <c r="D63" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E63" s="13" t="inlineStr">
+        <is>
+          <t>수리반환</t>
+        </is>
+      </c>
+      <c r="F63" s="176" t="n"/>
+      <c r="G63" s="177" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H63" s="16" t="n">
+        <v>400</v>
+      </c>
+      <c r="I63" s="178">
+        <f>IFERROR(VLOOKUP(B63,RemitTable2,7,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="J63" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K63" s="18">
+        <f>IFERROR(ROUND(H63*I63,0),0)</f>
+        <v/>
+      </c>
+      <c r="L63" s="18">
+        <f>IFERROR(VLOOKUP(B63,RemitTable2,10,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="M63" s="18">
+        <f>IFERROR(VLOOKUP(B63,RemitTable2,11,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N63" s="12" t="inlineStr">
+        <is>
+          <t>Display Card (수리반환 5PCS)</t>
+        </is>
+      </c>
+      <c r="O63" s="177" t="n">
+        <v>46125</v>
+      </c>
+      <c r="P63" s="12" t="inlineStr">
+        <is>
+          <t>22356-26-351613M</t>
+        </is>
+      </c>
+      <c r="Q63" s="16">
+        <f>IF(P63="","",IFERROR(VLOOKUP(O63,FxRateTable,4,TRUE),""))</f>
+        <v/>
+      </c>
+      <c r="R63" s="18">
+        <f>IF(P63="","",H63)</f>
+        <v/>
+      </c>
+      <c r="S63" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="T63" s="18" t="n">
+        <v>67750</v>
+      </c>
+      <c r="U63" s="13" t="n"/>
+      <c r="V63" s="12" t="inlineStr">
+        <is>
+          <t>운서합동</t>
+        </is>
+      </c>
+      <c r="W63" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="X63" s="13" t="inlineStr">
+        <is>
+          <t>DHL</t>
+        </is>
+      </c>
+      <c r="Y63" s="18" t="n">
+        <v>216006</v>
+      </c>
+      <c r="Z63" s="18">
+        <f>S63+T63+W63</f>
+        <v/>
+      </c>
+      <c r="AA63" s="18">
+        <f>K63+L63+M63+IFERROR(VLOOKUP(B63,RemitTable2,9,FALSE),0)+Y63+Z63</f>
+        <v/>
+      </c>
+      <c r="AB63" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="AC63" s="18">
+        <f>ROUND(AA63/AB63,0)</f>
+        <v/>
+      </c>
+      <c r="AD63" s="12" t="inlineStr">
+        <is>
           <t>2026-04</t>
         </is>
       </c>
-      <c r="AE62" s="177" t="n"/>
-      <c r="AF62" s="176" t="n"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="216" t="n">
+      <c r="AE63" s="177" t="n"/>
+      <c r="AF63" s="176" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="216" t="n">
         <v>59</v>
       </c>
-      <c r="B63" s="216" t="inlineStr">
+      <c r="B64" s="216" t="inlineStr">
         <is>
           <t>FRC-MONOPLEX26</t>
         </is>
       </c>
-      <c r="C63" s="217" t="inlineStr">
+      <c r="C64" s="217" t="inlineStr">
         <is>
           <t>Ferco</t>
         </is>
       </c>
-      <c r="D63" s="216" t="inlineStr">
+      <c r="D64" s="216" t="inlineStr">
         <is>
           <t>50% TT advance + 50% balance</t>
         </is>
       </c>
-      <c r="E63" s="217" t="inlineStr">
+      <c r="E64" s="217" t="inlineStr">
         <is>
           <t>기타</t>
         </is>
       </c>
-      <c r="F63" s="218" t="n">
+      <c r="F64" s="218" t="n">
         <v>46048</v>
       </c>
-      <c r="G63" s="219" t="n">
+      <c r="G64" s="219" t="n">
         <v>46133</v>
       </c>
-      <c r="H63" s="220" t="n">
+      <c r="H64" s="220" t="n">
         <v>51952</v>
       </c>
-      <c r="I63" s="221">
-        <f>IFERROR(VLOOKUP(B63,RemitTable2,7,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="J63" s="222" t="n">
-        <v>0</v>
-      </c>
-      <c r="K63" s="222">
-        <f>IFERROR(ROUND(H63*I63,0),0)</f>
-        <v/>
-      </c>
-      <c r="L63" s="222">
-        <f>IFERROR(VLOOKUP(B63,RemitTable2,10,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M63" s="222">
-        <f>IFERROR(VLOOKUP(B63,RemitTable2,11,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="N63" s="216" t="inlineStr">
+      <c r="I64" s="221">
+        <f>IFERROR(VLOOKUP(B64,RemitTable2,7,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="J64" s="222" t="n">
+        <v>0</v>
+      </c>
+      <c r="K64" s="222">
+        <f>IFERROR(ROUND(H64*I64,0),0)</f>
+        <v/>
+      </c>
+      <c r="L64" s="222">
+        <f>IFERROR(VLOOKUP(B64,RemitTable2,10,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="M64" s="222">
+        <f>IFERROR(VLOOKUP(B64,RemitTable2,11,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N64" s="216" t="inlineStr">
         <is>
           <t>Cinema Seat (Recliner) / 44 EA / Monoplex DH Bangbae</t>
         </is>
       </c>
-      <c r="O63" s="219" t="n">
+      <c r="O64" s="219" t="n">
         <v>46153</v>
       </c>
-      <c r="P63" s="216" t="inlineStr">
+      <c r="P64" s="216" t="inlineStr">
         <is>
           <t>14008-26-101147M</t>
         </is>
       </c>
-      <c r="Q63" s="220">
-        <f>IF(P63="","",IFERROR(VLOOKUP(O63,FxRateTable,4,TRUE),""))</f>
-        <v/>
-      </c>
-      <c r="R63" s="220">
-        <f>IF(P63="","",H63)</f>
-        <v/>
-      </c>
-      <c r="S63" s="222" t="n">
+      <c r="Q64" s="220">
+        <f>IF(P64="","",IFERROR(VLOOKUP(O64,FxRateTable,4,TRUE),""))</f>
+        <v/>
+      </c>
+      <c r="R64" s="220">
+        <f>IF(P64="","",H64)</f>
+        <v/>
+      </c>
+      <c r="S64" s="222" t="n">
         <v>31050</v>
       </c>
-      <c r="T63" s="222" t="n">
+      <c r="T64" s="222" t="n">
         <v>7959560</v>
       </c>
-      <c r="U63" s="218" t="n"/>
-      <c r="V63" s="216" t="inlineStr">
+      <c r="U64" s="218" t="n"/>
+      <c r="V64" s="216" t="inlineStr">
         <is>
           <t>조운관세사무소</t>
         </is>
       </c>
-      <c r="W63" s="222" t="n">
+      <c r="W64" s="222" t="n">
         <v>250000</v>
       </c>
-      <c r="X63" s="217" t="inlineStr">
+      <c r="X64" s="217" t="inlineStr">
         <is>
           <t>진로직스</t>
         </is>
       </c>
-      <c r="Y63" s="222" t="n">
+      <c r="Y64" s="222" t="n">
         <v>5002612</v>
       </c>
-      <c r="Z63" s="222">
-        <f>S63+T63+W63</f>
-        <v/>
-      </c>
-      <c r="AA63" s="222">
-        <f>K63+L63+M63+IFERROR(VLOOKUP(B63,RemitTable2,9,FALSE),0)+Y63+Z63</f>
-        <v/>
-      </c>
-      <c r="AB63" s="223" t="n">
+      <c r="Z64" s="222">
+        <f>S64+T64+W64</f>
+        <v/>
+      </c>
+      <c r="AA64" s="222">
+        <f>K64+L64+M64+IFERROR(VLOOKUP(B64,RemitTable2,9,FALSE),0)+Y64+Z64</f>
+        <v/>
+      </c>
+      <c r="AB64" s="223" t="n">
         <v>44</v>
       </c>
-      <c r="AC63" s="222">
-        <f>ROUND(AA63/AB63,0)</f>
-        <v/>
-      </c>
-      <c r="AD63" s="216" t="inlineStr">
+      <c r="AC64" s="222">
+        <f>ROUND(AA64/AB64,0)</f>
+        <v/>
+      </c>
+      <c r="AD64" s="216" t="inlineStr">
         <is>
           <t>2026-05</t>
         </is>
       </c>
-      <c r="AE63" s="216" t="n"/>
-      <c r="AF63" s="217" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="147" t="inlineStr">
-        <is>
-          <t>장비/부품 합계</t>
-        </is>
-      </c>
-      <c r="B64" s="148" t="n"/>
-      <c r="C64" s="148" t="n"/>
-      <c r="D64" s="148" t="n"/>
-      <c r="E64" s="148" t="n"/>
-      <c r="F64" s="148" t="n"/>
-      <c r="G64" s="149" t="n"/>
-      <c r="H64" s="142">
-        <f>SUBTOTAL(9,H5:H38)</f>
-        <v/>
-      </c>
-      <c r="I64" s="141" t="n"/>
-      <c r="J64" s="142">
-        <f>SUBTOTAL(9,J5:J38)</f>
-        <v/>
-      </c>
-      <c r="K64" s="142">
-        <f>SUBTOTAL(9,K5:K38)</f>
-        <v/>
-      </c>
-      <c r="L64" s="142">
-        <f>SUBTOTAL(9,L5:L38)</f>
-        <v/>
-      </c>
-      <c r="M64" s="142">
-        <f>SUBTOTAL(9,M5:M38)</f>
-        <v/>
-      </c>
-      <c r="N64" s="141" t="n"/>
-      <c r="O64" s="141" t="n"/>
-      <c r="P64" s="141" t="n"/>
-      <c r="Q64" s="142" t="n"/>
-      <c r="R64" s="140" t="n"/>
-      <c r="S64" s="142">
-        <f>SUBTOTAL(9,S5:S38)</f>
-        <v/>
-      </c>
-      <c r="T64" s="142">
-        <f>SUBTOTAL(9,T5:T38)</f>
-        <v/>
-      </c>
-      <c r="U64" s="141" t="n"/>
-      <c r="V64" s="141" t="n"/>
-      <c r="W64" s="142">
-        <f>SUBTOTAL(9,W5:W38)</f>
-        <v/>
-      </c>
-      <c r="X64" s="147" t="n"/>
-      <c r="Y64" s="142">
-        <f>SUBTOTAL(9,Y5:Y38)</f>
-        <v/>
-      </c>
-      <c r="Z64" s="142">
-        <f>SUBTOTAL(9,Z5:Z38)</f>
-        <v/>
-      </c>
-      <c r="AA64" s="142">
-        <f>SUBTOTAL(9,AA5:AA38)</f>
-        <v/>
-      </c>
-      <c r="AB64" s="147" t="n"/>
-      <c r="AC64" s="141" t="n"/>
-      <c r="AD64" s="141" t="n"/>
-      <c r="AE64" s="141" t="n"/>
-      <c r="AF64" s="141" t="n"/>
+      <c r="AE64" s="216" t="n"/>
+      <c r="AF64" s="217" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="147" t="inlineStr">
         <is>
-          <t>라이센스/워런티 합계</t>
+          <t>장비/부품 합계</t>
         </is>
       </c>
       <c r="B65" s="148" t="n"/>
@@ -9386,24 +9455,24 @@
       <c r="F65" s="148" t="n"/>
       <c r="G65" s="149" t="n"/>
       <c r="H65" s="142">
-        <f>SUBTOTAL(9,H39:H60)</f>
+        <f>SUBTOTAL(9,H5:H39)</f>
         <v/>
       </c>
       <c r="I65" s="141" t="n"/>
       <c r="J65" s="142">
-        <f>SUBTOTAL(9,J39:J60)</f>
+        <f>SUBTOTAL(9,J5:J39)</f>
         <v/>
       </c>
       <c r="K65" s="142">
-        <f>SUBTOTAL(9,K39:K60)</f>
+        <f>SUBTOTAL(9,K5:K39)</f>
         <v/>
       </c>
       <c r="L65" s="142">
-        <f>SUBTOTAL(9,L39:L60)</f>
+        <f>SUBTOTAL(9,L5:L39)</f>
         <v/>
       </c>
       <c r="M65" s="142">
-        <f>SUBTOTAL(9,M39:M60)</f>
+        <f>SUBTOTAL(9,M5:M39)</f>
         <v/>
       </c>
       <c r="N65" s="141" t="n"/>
@@ -9412,30 +9481,30 @@
       <c r="Q65" s="142" t="n"/>
       <c r="R65" s="140" t="n"/>
       <c r="S65" s="142">
-        <f>SUBTOTAL(9,S39:S60)</f>
+        <f>SUBTOTAL(9,S5:S39)</f>
         <v/>
       </c>
       <c r="T65" s="142">
-        <f>SUBTOTAL(9,T39:T60)</f>
+        <f>SUBTOTAL(9,T5:T39)</f>
         <v/>
       </c>
       <c r="U65" s="141" t="n"/>
       <c r="V65" s="141" t="n"/>
       <c r="W65" s="142">
-        <f>SUBTOTAL(9,W39:W60)</f>
+        <f>SUBTOTAL(9,W5:W39)</f>
         <v/>
       </c>
       <c r="X65" s="147" t="n"/>
       <c r="Y65" s="142">
-        <f>SUBTOTAL(9,Y39:Y60)</f>
+        <f>SUBTOTAL(9,Y5:Y39)</f>
         <v/>
       </c>
       <c r="Z65" s="142">
-        <f>SUBTOTAL(9,Z39:Z60)</f>
+        <f>SUBTOTAL(9,Z5:Z39)</f>
         <v/>
       </c>
       <c r="AA65" s="142">
-        <f>SUBTOTAL(9,AA39:AA60)</f>
+        <f>SUBTOTAL(9,AA5:AA39)</f>
         <v/>
       </c>
       <c r="AB65" s="147" t="n"/>
@@ -9447,7 +9516,7 @@
     <row r="66">
       <c r="A66" s="147" t="inlineStr">
         <is>
-          <t>기타 합계</t>
+          <t>라이센스/워런티 합계</t>
         </is>
       </c>
       <c r="B66" s="148" t="n"/>
@@ -9457,24 +9526,24 @@
       <c r="F66" s="148" t="n"/>
       <c r="G66" s="149" t="n"/>
       <c r="H66" s="142">
-        <f>SUBTOTAL(9,H61:H63)</f>
+        <f>SUBTOTAL(9,H40:H61)</f>
         <v/>
       </c>
       <c r="I66" s="141" t="n"/>
       <c r="J66" s="142">
-        <f>SUBTOTAL(9,J61:J63)</f>
+        <f>SUBTOTAL(9,J40:J61)</f>
         <v/>
       </c>
       <c r="K66" s="142">
-        <f>SUBTOTAL(9,K61:K63)</f>
+        <f>SUBTOTAL(9,K40:K61)</f>
         <v/>
       </c>
       <c r="L66" s="142">
-        <f>SUBTOTAL(9,L61:L63)</f>
+        <f>SUBTOTAL(9,L40:L61)</f>
         <v/>
       </c>
       <c r="M66" s="142">
-        <f>SUBTOTAL(9,M61:M63)</f>
+        <f>SUBTOTAL(9,M40:M61)</f>
         <v/>
       </c>
       <c r="N66" s="141" t="n"/>
@@ -9483,30 +9552,30 @@
       <c r="Q66" s="142" t="n"/>
       <c r="R66" s="140" t="n"/>
       <c r="S66" s="142">
-        <f>SUBTOTAL(9,S61:S63)</f>
+        <f>SUBTOTAL(9,S40:S61)</f>
         <v/>
       </c>
       <c r="T66" s="142">
-        <f>SUBTOTAL(9,T61:T63)</f>
+        <f>SUBTOTAL(9,T40:T61)</f>
         <v/>
       </c>
       <c r="U66" s="141" t="n"/>
       <c r="V66" s="141" t="n"/>
       <c r="W66" s="142">
-        <f>SUBTOTAL(9,W61:W63)</f>
+        <f>SUBTOTAL(9,W40:W61)</f>
         <v/>
       </c>
       <c r="X66" s="147" t="n"/>
       <c r="Y66" s="142">
-        <f>SUBTOTAL(9,Y61:Y63)</f>
+        <f>SUBTOTAL(9,Y40:Y61)</f>
         <v/>
       </c>
       <c r="Z66" s="142">
-        <f>SUBTOTAL(9,Z61:Z63)</f>
+        <f>SUBTOTAL(9,Z40:Z61)</f>
         <v/>
       </c>
       <c r="AA66" s="142">
-        <f>SUBTOTAL(9,AA61:AA63)</f>
+        <f>SUBTOTAL(9,AA40:AA61)</f>
         <v/>
       </c>
       <c r="AB66" s="147" t="n"/>
@@ -9516,9 +9585,9 @@
       <c r="AF66" s="141" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="154" t="inlineStr">
-        <is>
-          <t>총 합계</t>
+      <c r="A67" s="147" t="inlineStr">
+        <is>
+          <t>기타 합계</t>
         </is>
       </c>
       <c r="B67" s="148" t="n"/>
@@ -9527,98 +9596,135 @@
       <c r="E67" s="148" t="n"/>
       <c r="F67" s="148" t="n"/>
       <c r="G67" s="149" t="n"/>
-      <c r="H67" s="146">
-        <f>SUBTOTAL(9,H5:H63)</f>
-        <v/>
-      </c>
-      <c r="I67" s="145" t="n"/>
-      <c r="J67" s="146">
-        <f>SUBTOTAL(9,J5:J63)</f>
-        <v/>
-      </c>
-      <c r="K67" s="146">
-        <f>SUBTOTAL(9,K5:K63)</f>
-        <v/>
-      </c>
-      <c r="L67" s="146">
-        <f>SUBTOTAL(9,L5:L63)</f>
-        <v/>
-      </c>
-      <c r="M67" s="146">
-        <f>SUBTOTAL(9,M5:M63)</f>
-        <v/>
-      </c>
-      <c r="N67" s="145" t="n"/>
-      <c r="O67" s="145" t="n"/>
-      <c r="P67" s="145" t="n"/>
-      <c r="Q67" s="146" t="n"/>
-      <c r="R67" s="144" t="n"/>
-      <c r="S67" s="146">
-        <f>SUBTOTAL(9,S5:S63)</f>
-        <v/>
-      </c>
-      <c r="T67" s="146">
-        <f>SUBTOTAL(9,T5:T63)</f>
-        <v/>
-      </c>
-      <c r="U67" s="145" t="n"/>
-      <c r="V67" s="145" t="n"/>
-      <c r="W67" s="146">
-        <f>SUBTOTAL(9,W5:W63)</f>
-        <v/>
-      </c>
-      <c r="X67" s="154" t="n"/>
-      <c r="Y67" s="146">
-        <f>SUBTOTAL(9,Y5:Y63)</f>
-        <v/>
-      </c>
-      <c r="Z67" s="146">
-        <f>SUBTOTAL(9,Z5:Z63)</f>
-        <v/>
-      </c>
-      <c r="AA67" s="146">
-        <f>SUBTOTAL(9,AA5:AA63)</f>
-        <v/>
-      </c>
-      <c r="AB67" s="154" t="n"/>
-      <c r="AC67" s="145" t="n"/>
-      <c r="AD67" s="145" t="n"/>
-      <c r="AE67" s="145" t="n"/>
-      <c r="AF67" s="145" t="n"/>
+      <c r="H67" s="142">
+        <f>SUBTOTAL(9,H62:H64)</f>
+        <v/>
+      </c>
+      <c r="I67" s="141" t="n"/>
+      <c r="J67" s="142">
+        <f>SUBTOTAL(9,J62:J64)</f>
+        <v/>
+      </c>
+      <c r="K67" s="142">
+        <f>SUBTOTAL(9,K62:K64)</f>
+        <v/>
+      </c>
+      <c r="L67" s="142">
+        <f>SUBTOTAL(9,L62:L64)</f>
+        <v/>
+      </c>
+      <c r="M67" s="142">
+        <f>SUBTOTAL(9,M62:M64)</f>
+        <v/>
+      </c>
+      <c r="N67" s="141" t="n"/>
+      <c r="O67" s="141" t="n"/>
+      <c r="P67" s="141" t="n"/>
+      <c r="Q67" s="142" t="n"/>
+      <c r="R67" s="140" t="n"/>
+      <c r="S67" s="142">
+        <f>SUBTOTAL(9,S62:S64)</f>
+        <v/>
+      </c>
+      <c r="T67" s="142">
+        <f>SUBTOTAL(9,T62:T64)</f>
+        <v/>
+      </c>
+      <c r="U67" s="141" t="n"/>
+      <c r="V67" s="141" t="n"/>
+      <c r="W67" s="142">
+        <f>SUBTOTAL(9,W62:W64)</f>
+        <v/>
+      </c>
+      <c r="X67" s="147" t="n"/>
+      <c r="Y67" s="142">
+        <f>SUBTOTAL(9,Y62:Y64)</f>
+        <v/>
+      </c>
+      <c r="Z67" s="142">
+        <f>SUBTOTAL(9,Z62:Z64)</f>
+        <v/>
+      </c>
+      <c r="AA67" s="142">
+        <f>SUBTOTAL(9,AA62:AA64)</f>
+        <v/>
+      </c>
+      <c r="AB67" s="147" t="n"/>
+      <c r="AC67" s="141" t="n"/>
+      <c r="AD67" s="141" t="n"/>
+      <c r="AE67" s="141" t="n"/>
+      <c r="AF67" s="141" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="39" t="n"/>
-      <c r="B68" s="39" t="n"/>
-      <c r="C68" s="39" t="n"/>
-      <c r="D68" s="39" t="n"/>
-      <c r="E68" s="39" t="n"/>
-      <c r="F68" s="39" t="n"/>
-      <c r="G68" s="39" t="n"/>
-      <c r="H68" s="39" t="n"/>
-      <c r="I68" s="39" t="n"/>
-      <c r="J68" s="39" t="n"/>
-      <c r="K68" s="39" t="n"/>
-      <c r="L68" s="39" t="n"/>
-      <c r="M68" s="39" t="n"/>
-      <c r="N68" s="39" t="n"/>
-      <c r="O68" s="39" t="n"/>
-      <c r="P68" s="39" t="n"/>
-      <c r="Q68" s="39" t="n"/>
-      <c r="R68" s="39" t="n"/>
-      <c r="S68" s="39" t="n"/>
-      <c r="T68" s="39" t="n"/>
-      <c r="U68" s="39" t="n"/>
-      <c r="V68" s="39" t="n"/>
-      <c r="W68" s="39" t="n"/>
-      <c r="X68" s="75" t="n"/>
-      <c r="Y68" s="39" t="n"/>
-      <c r="Z68" s="39" t="n"/>
-      <c r="AA68" s="39" t="n"/>
-      <c r="AB68" s="75" t="n"/>
-      <c r="AC68" s="39" t="n"/>
-      <c r="AD68" s="39" t="n"/>
-      <c r="AE68" s="39" t="n"/>
-      <c r="AF68" s="39" t="n"/>
+      <c r="A68" s="154" t="inlineStr">
+        <is>
+          <t>총 합계</t>
+        </is>
+      </c>
+      <c r="B68" s="148" t="n"/>
+      <c r="C68" s="148" t="n"/>
+      <c r="D68" s="148" t="n"/>
+      <c r="E68" s="148" t="n"/>
+      <c r="F68" s="148" t="n"/>
+      <c r="G68" s="149" t="n"/>
+      <c r="H68" s="146">
+        <f>SUBTOTAL(9,H5:H64)</f>
+        <v/>
+      </c>
+      <c r="I68" s="145" t="n"/>
+      <c r="J68" s="146">
+        <f>SUBTOTAL(9,J5:J64)</f>
+        <v/>
+      </c>
+      <c r="K68" s="146">
+        <f>SUBTOTAL(9,K5:K64)</f>
+        <v/>
+      </c>
+      <c r="L68" s="146">
+        <f>SUBTOTAL(9,L5:L64)</f>
+        <v/>
+      </c>
+      <c r="M68" s="146">
+        <f>SUBTOTAL(9,M5:M64)</f>
+        <v/>
+      </c>
+      <c r="N68" s="145" t="n"/>
+      <c r="O68" s="145" t="n"/>
+      <c r="P68" s="145" t="n"/>
+      <c r="Q68" s="146" t="n"/>
+      <c r="R68" s="144" t="n"/>
+      <c r="S68" s="146">
+        <f>SUBTOTAL(9,S5:S64)</f>
+        <v/>
+      </c>
+      <c r="T68" s="146">
+        <f>SUBTOTAL(9,T5:T64)</f>
+        <v/>
+      </c>
+      <c r="U68" s="145" t="n"/>
+      <c r="V68" s="145" t="n"/>
+      <c r="W68" s="146">
+        <f>SUBTOTAL(9,W5:W64)</f>
+        <v/>
+      </c>
+      <c r="X68" s="154" t="n"/>
+      <c r="Y68" s="146">
+        <f>SUBTOTAL(9,Y5:Y64)</f>
+        <v/>
+      </c>
+      <c r="Z68" s="146">
+        <f>SUBTOTAL(9,Z5:Z64)</f>
+        <v/>
+      </c>
+      <c r="AA68" s="146">
+        <f>SUBTOTAL(9,AA5:AA64)</f>
+        <v/>
+      </c>
+      <c r="AB68" s="154" t="n"/>
+      <c r="AC68" s="145" t="n"/>
+      <c r="AD68" s="145" t="n"/>
+      <c r="AE68" s="145" t="n"/>
+      <c r="AF68" s="145" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="39" t="n"/>
@@ -9756,8 +9862,42 @@
       <c r="AE72" s="39" t="n"/>
       <c r="AF72" s="39" t="n"/>
     </row>
-    <row r="86">
-      <c r="M86" s="40" t="n"/>
+    <row r="73">
+      <c r="A73" s="39" t="n"/>
+      <c r="B73" s="39" t="n"/>
+      <c r="C73" s="39" t="n"/>
+      <c r="D73" s="39" t="n"/>
+      <c r="E73" s="39" t="n"/>
+      <c r="F73" s="39" t="n"/>
+      <c r="G73" s="39" t="n"/>
+      <c r="H73" s="39" t="n"/>
+      <c r="I73" s="39" t="n"/>
+      <c r="J73" s="39" t="n"/>
+      <c r="K73" s="39" t="n"/>
+      <c r="L73" s="39" t="n"/>
+      <c r="M73" s="39" t="n"/>
+      <c r="N73" s="39" t="n"/>
+      <c r="O73" s="39" t="n"/>
+      <c r="P73" s="39" t="n"/>
+      <c r="Q73" s="39" t="n"/>
+      <c r="R73" s="39" t="n"/>
+      <c r="S73" s="39" t="n"/>
+      <c r="T73" s="39" t="n"/>
+      <c r="U73" s="39" t="n"/>
+      <c r="V73" s="39" t="n"/>
+      <c r="W73" s="39" t="n"/>
+      <c r="X73" s="75" t="n"/>
+      <c r="Y73" s="39" t="n"/>
+      <c r="Z73" s="39" t="n"/>
+      <c r="AA73" s="39" t="n"/>
+      <c r="AB73" s="75" t="n"/>
+      <c r="AC73" s="39" t="n"/>
+      <c r="AD73" s="39" t="n"/>
+      <c r="AE73" s="39" t="n"/>
+      <c r="AF73" s="39" t="n"/>
+    </row>
+    <row r="87">
+      <c r="M87" s="40" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -9767,9 +9907,9 @@
     <mergeCell ref="A1:AF1"/>
     <mergeCell ref="AD3:AF3"/>
     <mergeCell ref="X3:Z3"/>
-    <mergeCell ref="A64:G64"/>
     <mergeCell ref="A65:G65"/>
     <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A68:G68"/>
     <mergeCell ref="AA3:AC3"/>
     <mergeCell ref="O3:W3"/>
     <mergeCell ref="A2:AF2"/>
@@ -12413,11 +12553,11 @@
       </c>
       <c r="G34" s="241" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>DHL</t>
         </is>
       </c>
       <c r="H34" s="244" t="n">
-        <v>0</v>
+        <v>216006</v>
       </c>
       <c r="I34" s="241" t="inlineStr">
         <is>
@@ -12461,7 +12601,7 @@
         </is>
       </c>
       <c r="H35" s="244" t="n">
-        <v>0</v>
+        <v>174806</v>
       </c>
       <c r="I35" s="241" t="inlineStr">
         <is>

</xml_diff>